<commit_message>
USB swap and updated BOM
</commit_message>
<xml_diff>
--- a/2025-2026_Boards/FDCAN-USB_Board/Manufacturing/JLCPCB_BOM_FDCAN-USB_Board.xlsx
+++ b/2025-2026_Boards/FDCAN-USB_Board/Manufacturing/JLCPCB_BOM_FDCAN-USB_Board.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dawso\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dawso\Desktop\MarsRover\KiCad\2025-2026_Boards\FDCAN-USB_Board\Manufacturing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D35721-BDD7-4077-A18B-AF0ED0F54FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A6F7157-1920-4870-A8EC-E2EDC7076C02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="1740" windowWidth="14610" windowHeight="15585" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -103,9 +103,6 @@
     <t>LED_SMD:LED_0603_1608Metric</t>
   </si>
   <si>
-    <t>USB4110-GF-A_GCT</t>
-  </si>
-  <si>
     <t>JST_PH_S3B-PH-SM4-TB_1x03-1MP_P2.00mm_Horizontal</t>
   </si>
   <si>
@@ -142,18 +139,6 @@
     <t>USBLC6-2SC6</t>
   </si>
   <si>
-    <t>TCAN1057AEV-Q1</t>
-  </si>
-  <si>
-    <t>BD120-10-A-0305-0229-L-B</t>
-  </si>
-  <si>
-    <t>C17362550</t>
-  </si>
-  <si>
-    <t>C5143397</t>
-  </si>
-  <si>
     <t>C347222</t>
   </si>
   <si>
@@ -166,9 +151,6 @@
     <t>STM32G474CET6</t>
   </si>
   <si>
-    <t>C22458650</t>
-  </si>
-  <si>
     <t>C265101</t>
   </si>
   <si>
@@ -223,9 +205,6 @@
     <t>Yellow, Lite-On LTST-C193KSKT-5A</t>
   </si>
   <si>
-    <t xml:space="preserve">USB4110-GF-A </t>
-  </si>
-  <si>
     <t>Green, Lite-On LTST-C193KGKT-5A</t>
   </si>
   <si>
@@ -257,6 +236,27 @@
   </si>
   <si>
     <t>C112291</t>
+  </si>
+  <si>
+    <t>C3234997</t>
+  </si>
+  <si>
+    <t>HX PZ1.27-2x5P ZZ, hanxia</t>
+  </si>
+  <si>
+    <t>C22438120</t>
+  </si>
+  <si>
+    <t>TCAN1057AEVDRQ1</t>
+  </si>
+  <si>
+    <t>2171790001, Molex</t>
+  </si>
+  <si>
+    <t>C3197684</t>
+  </si>
+  <si>
+    <t>2171790001_MOL</t>
   </si>
 </sst>
 </file>
@@ -718,7 +718,7 @@
     </row>
     <row r="2" spans="1:4" ht="19.95" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>3</v>
@@ -727,12 +727,12 @@
         <v>23</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="19.95" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>5</v>
@@ -741,26 +741,26 @@
         <v>23</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="19.95" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>6</v>
@@ -769,12 +769,12 @@
         <v>24</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="19.95" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
@@ -783,12 +783,12 @@
         <v>25</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="19.95" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>8</v>
@@ -797,12 +797,12 @@
         <v>26</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="19.95" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>9</v>
@@ -811,12 +811,12 @@
         <v>26</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="19.95" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>10</v>
@@ -825,12 +825,12 @@
         <v>26</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="19.95" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>11</v>
@@ -839,161 +839,161 @@
         <v>26</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="19.95" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="19.95" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="19.95" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="19.95" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="19.95" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="19.95" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="19.95" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="19.95" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="19.95" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="19.95" customHeight="1">
       <c r="A20" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="19.95" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>